<commit_message>
Add GEO brand fact knowledge base
</commit_message>
<xml_diff>
--- a/public/downloads/yhl-geo-90-day-content-execution.xlsx
+++ b/public/downloads/yhl-geo-90-day-content-execution.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容总矩阵" sheetId="1" r:id="R121384d16dfa41d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面规格" sheetId="2" r:id="R67ab1dadf77d4177"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ计划" sheetId="3" r:id="Rcc66e11cc79d439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="信源补强" sheetId="4" r:id="Rdb15a15839b84b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90天排期" sheetId="5" r:id="R5379fa9f162949f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI看板" sheetId="6" r:id="Rea3f5c6ad6c54838"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布质检" sheetId="7" r:id="Re06e9beb197b4f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="内容总矩阵" sheetId="1" r:id="Rd97f256f8c884e6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面规格" sheetId="2" r:id="R89f614f2bfa54a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ计划" sheetId="3" r:id="R8ea4aa6125b84c9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="信源补强" sheetId="4" r:id="Rf8affba3d97942a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="90天排期" sheetId="5" r:id="R64b3663fbb404d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI看板" sheetId="6" r:id="R7d0ab3dd4a074c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发布质检" sheetId="7" r:id="Rba21dea103b74c2b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{4E667B02-A865-4B47-8DA4-55B6D82F43E8}"/>
+  <xltc:person displayName="User" id="{7A661B72-46B1-4170-B73B-BDA9A377787C}"/>
 </xltc:personList>
 </file>
 
@@ -611,7 +611,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Roadmap90Table" displayName="Roadmap90Table" ref="A4:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Roadmap90Table" displayName="Roadmap90Table" ref="A4:L24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="task_id"/>
     <x:tableColumn id="2" name="阶段"/>
@@ -631,7 +631,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="KpiTable" displayName="KpiTable" ref="A4:J17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="KpiTable" displayName="KpiTable" ref="A4:J21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="指标层"/>
     <x:tableColumn id="2" name="指标"/>
@@ -649,7 +649,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PublishQATable" displayName="PublishQATable" ref="A4:K52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PublishQATable" displayName="PublishQATable" ref="A4:K58" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="check_id"/>
     <x:tableColumn id="2" name="资产"/>
@@ -2463,7 +2463,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3af46a6584ad483c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c136ee665284010"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3317,7 +3317,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf26f8314f91243ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R576dedbadc52414c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3984,7 +3984,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2c32d5bcbbd47e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78f9231cefc64f27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5441,7 +5441,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re867047e373e4c71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59f55b7a215245fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5705,495 +5705,571 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="45" t="str">
-        <x:v>T-006</x:v>
+        <x:v>T-KB-001</x:v>
       </x:c>
       <x:c r="B10" s="46" t="str">
         <x:v>0-30天 事实基础</x:v>
       </x:c>
       <x:c r="C10" s="46" t="str">
-        <x:v>D10-D25</x:v>
+        <x:v>D15-D22</x:v>
       </x:c>
       <x:c r="D10" s="46" t="str">
-        <x:v>补3条待核验信源的原文或交叉来源</x:v>
+        <x:v>建立11表品牌事实知识库与公开JSON</x:v>
       </x:c>
       <x:c r="E10" s="46" t="str">
-        <x:v>信源补强</x:v>
+        <x:v>独立知识库+公开快照JSON+网站入口</x:v>
       </x:c>
       <x:c r="F10" s="46" t="str">
-        <x:v>外部原始页面</x:v>
+        <x:v>信源库/FAQ/证据索引</x:v>
       </x:c>
       <x:c r="G10" s="46" t="str">
-        <x:v>信源核验</x:v>
+        <x:v>数据QA+信源核验</x:v>
       </x:c>
       <x:c r="H10" s="46" t="str">
-        <x:v>27/27状态明确</x:v>
+        <x:v>27条信源、30题、15FAQ全部映射</x:v>
       </x:c>
       <x:c r="I10" s="55" t="n">
-        <x:v>46230</x:v>
+        <x:v>46234</x:v>
       </x:c>
       <x:c r="J10" s="55" t="n">
-        <x:v>46245</x:v>
+        <x:v>46241</x:v>
       </x:c>
       <x:c r="K10" s="58" t="str">
-        <x:v>待开始</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="L10" s="47" t="str">
-        <x:v>不阻塞投递</x:v>
+        <x:v>不合并进执行大表</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="45" t="str">
-        <x:v>T-007</x:v>
+        <x:v>T-006</x:v>
       </x:c>
       <x:c r="B11" s="46" t="str">
         <x:v>0-30天 事实基础</x:v>
       </x:c>
       <x:c r="C11" s="46" t="str">
-        <x:v>D20-D30</x:v>
+        <x:v>D10-D25</x:v>
       </x:c>
       <x:c r="D11" s="46" t="str">
-        <x:v>完成页面、下载、robots、sitemap和移动端质检</x:v>
+        <x:v>补3条待核验信源的原文或交叉来源</x:v>
       </x:c>
       <x:c r="E11" s="46" t="str">
-        <x:v>发布质检记录</x:v>
+        <x:v>信源补强</x:v>
       </x:c>
       <x:c r="F11" s="46" t="str">
-        <x:v>网站部署</x:v>
+        <x:v>外部原始页面</x:v>
       </x:c>
       <x:c r="G11" s="46" t="str">
-        <x:v>数据QA+网站编辑</x:v>
+        <x:v>信源核验</x:v>
       </x:c>
       <x:c r="H11" s="46" t="str">
-        <x:v>所有硬验收通过</x:v>
+        <x:v>27/27状态明确</x:v>
       </x:c>
       <x:c r="I11" s="55" t="n">
-        <x:v>46239</x:v>
+        <x:v>46230</x:v>
       </x:c>
       <x:c r="J11" s="55" t="n">
-        <x:v>46249</x:v>
+        <x:v>46245</x:v>
       </x:c>
       <x:c r="K11" s="58" t="str">
-        <x:v>执行中</x:v>
+        <x:v>待开始</x:v>
       </x:c>
       <x:c r="L11" s="47" t="str">
-        <x:v>公开链接最终确认</x:v>
+        <x:v>不阻塞投递</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="45" t="str">
-        <x:v>T-008</x:v>
+        <x:v>T-007</x:v>
       </x:c>
       <x:c r="B12" s="46" t="str">
-        <x:v>31-60天 解释差异</x:v>
+        <x:v>0-30天 事实基础</x:v>
       </x:c>
       <x:c r="C12" s="46" t="str">
-        <x:v>D31-D36</x:v>
+        <x:v>D20-D30</x:v>
       </x:c>
       <x:c r="D12" s="46" t="str">
-        <x:v>评估品牌定位页拆分条件</x:v>
+        <x:v>完成页面、下载、robots、sitemap和移动端质检</x:v>
       </x:c>
       <x:c r="E12" s="46" t="str">
-        <x:v>拆页评审记录</x:v>
+        <x:v>发布质检记录</x:v>
       </x:c>
       <x:c r="F12" s="46" t="str">
-        <x:v>第三方定位证据</x:v>
+        <x:v>网站部署</x:v>
       </x:c>
       <x:c r="G12" s="46" t="str">
-        <x:v>内容策略+信源核验</x:v>
+        <x:v>数据QA+网站编辑</x:v>
       </x:c>
       <x:c r="H12" s="46" t="str">
-        <x:v>满足条件才拆页</x:v>
+        <x:v>所有硬验收通过</x:v>
       </x:c>
       <x:c r="I12" s="55" t="n">
-        <x:v>46250</x:v>
+        <x:v>46239</x:v>
       </x:c>
       <x:c r="J12" s="55" t="n">
-        <x:v>46255</x:v>
+        <x:v>46249</x:v>
       </x:c>
       <x:c r="K12" s="58" t="str">
-        <x:v>待开始</x:v>
+        <x:v>执行中</x:v>
       </x:c>
       <x:c r="L12" s="47" t="str">
-        <x:v>证据不足则维持合并</x:v>
+        <x:v>公开链接最终确认</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="45" t="str">
-        <x:v>T-009</x:v>
+        <x:v>T-008</x:v>
       </x:c>
       <x:c r="B13" s="46" t="str">
         <x:v>31-60天 解释差异</x:v>
       </x:c>
       <x:c r="C13" s="46" t="str">
-        <x:v>D34-D45</x:v>
+        <x:v>D31-D36</x:v>
       </x:c>
       <x:c r="D13" s="46" t="str">
-        <x:v>制作明式/清式风格指南</x:v>
+        <x:v>评估品牌定位页拆分条件</x:v>
       </x:c>
       <x:c r="E13" s="46" t="str">
-        <x:v>P1风格页面</x:v>
+        <x:v>拆页评审记录</x:v>
       </x:c>
       <x:c r="F13" s="46" t="str">
-        <x:v>博物馆/权威书目</x:v>
+        <x:v>第三方定位证据</x:v>
       </x:c>
       <x:c r="G13" s="46" t="str">
-        <x:v>内容策略</x:v>
+        <x:v>内容策略+信源核验</x:v>
       </x:c>
       <x:c r="H13" s="46" t="str">
-        <x:v>背景与产品证据分开</x:v>
+        <x:v>满足条件才拆页</x:v>
       </x:c>
       <x:c r="I13" s="55" t="n">
-        <x:v>46253</x:v>
+        <x:v>46250</x:v>
       </x:c>
       <x:c r="J13" s="55" t="n">
-        <x:v>46264</x:v>
+        <x:v>46255</x:v>
       </x:c>
       <x:c r="K13" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L13" s="47" t="str">
-        <x:v>不推断年代馆藏</x:v>
+        <x:v>证据不足则维持合并</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="45" t="str">
-        <x:v>T-010</x:v>
+        <x:v>T-009</x:v>
       </x:c>
       <x:c r="B14" s="46" t="str">
         <x:v>31-60天 解释差异</x:v>
       </x:c>
       <x:c r="C14" s="46" t="str">
-        <x:v>D38-D50</x:v>
+        <x:v>D34-D45</x:v>
       </x:c>
       <x:c r="D14" s="46" t="str">
-        <x:v>制作黄花梨/紫檀/酸枝专题</x:v>
+        <x:v>制作明式/清式风格指南</x:v>
       </x:c>
       <x:c r="E14" s="46" t="str">
-        <x:v>3个材质专题</x:v>
+        <x:v>P1风格页面</x:v>
       </x:c>
       <x:c r="F14" s="46" t="str">
-        <x:v>国家标准</x:v>
+        <x:v>博物馆/权威书目</x:v>
       </x:c>
       <x:c r="G14" s="46" t="str">
-        <x:v>信源核验+网站编辑</x:v>
+        <x:v>内容策略</x:v>
       </x:c>
       <x:c r="H14" s="46" t="str">
-        <x:v>术语/品牌/单件三层</x:v>
+        <x:v>背景与产品证据分开</x:v>
       </x:c>
       <x:c r="I14" s="55" t="n">
-        <x:v>46257</x:v>
+        <x:v>46253</x:v>
       </x:c>
       <x:c r="J14" s="55" t="n">
-        <x:v>46269</x:v>
+        <x:v>46264</x:v>
       </x:c>
       <x:c r="K14" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L14" s="47" t="str">
-        <x:v>可分批上线</x:v>
+        <x:v>不推断年代馆藏</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="45" t="str">
-        <x:v>T-011</x:v>
+        <x:v>T-010</x:v>
       </x:c>
       <x:c r="B15" s="46" t="str">
         <x:v>31-60天 解释差异</x:v>
       </x:c>
       <x:c r="C15" s="46" t="str">
-        <x:v>D42-D54</x:v>
+        <x:v>D38-D50</x:v>
       </x:c>
       <x:c r="D15" s="46" t="str">
-        <x:v>制作单件产品证据模板</x:v>
+        <x:v>制作黄花梨/紫檀/酸枝专题</x:v>
       </x:c>
       <x:c r="E15" s="46" t="str">
-        <x:v>产品证据模板</x:v>
+        <x:v>3个材质专题</x:v>
       </x:c>
       <x:c r="F15" s="46" t="str">
-        <x:v>合同/证书字段</x:v>
+        <x:v>国家标准</x:v>
       </x:c>
       <x:c r="G15" s="46" t="str">
-        <x:v>数据QA+网站编辑</x:v>
+        <x:v>信源核验+网站编辑</x:v>
       </x:c>
       <x:c r="H15" s="46" t="str">
-        <x:v>字段可复用</x:v>
+        <x:v>术语/品牌/单件三层</x:v>
       </x:c>
       <x:c r="I15" s="55" t="n">
-        <x:v>46261</x:v>
+        <x:v>46257</x:v>
       </x:c>
       <x:c r="J15" s="55" t="n">
-        <x:v>46273</x:v>
+        <x:v>46269</x:v>
       </x:c>
       <x:c r="K15" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L15" s="47" t="str">
-        <x:v>使用脱敏样例</x:v>
+        <x:v>可分批上线</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="45" t="str">
-        <x:v>T-012</x:v>
+        <x:v>T-011</x:v>
       </x:c>
       <x:c r="B16" s="46" t="str">
         <x:v>31-60天 解释差异</x:v>
       </x:c>
       <x:c r="C16" s="46" t="str">
-        <x:v>D46-D60</x:v>
+        <x:v>D42-D54</x:v>
       </x:c>
       <x:c r="D16" s="46" t="str">
-        <x:v>补全P1内链、元数据和结构化数据</x:v>
+        <x:v>制作单件产品证据模板</x:v>
       </x:c>
       <x:c r="E16" s="46" t="str">
-        <x:v>P1发布包</x:v>
+        <x:v>产品证据模板</x:v>
       </x:c>
       <x:c r="F16" s="46" t="str">
-        <x:v>P1页面</x:v>
+        <x:v>合同/证书字段</x:v>
       </x:c>
       <x:c r="G16" s="46" t="str">
-        <x:v>网站编辑</x:v>
+        <x:v>数据QA+网站编辑</x:v>
       </x:c>
       <x:c r="H16" s="46" t="str">
-        <x:v>无孤立页、无失效内链</x:v>
+        <x:v>字段可复用</x:v>
       </x:c>
       <x:c r="I16" s="55" t="n">
-        <x:v>46265</x:v>
+        <x:v>46261</x:v>
       </x:c>
       <x:c r="J16" s="55" t="n">
-        <x:v>46279</x:v>
+        <x:v>46273</x:v>
       </x:c>
       <x:c r="K16" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L16" s="47" t="str">
-        <x:v>发布前质检</x:v>
+        <x:v>使用脱敏样例</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="45" t="str">
-        <x:v>T-013</x:v>
+        <x:v>T-012</x:v>
       </x:c>
       <x:c r="B17" s="46" t="str">
-        <x:v>61-90天 复测维护</x:v>
+        <x:v>31-60天 解释差异</x:v>
       </x:c>
       <x:c r="C17" s="46" t="str">
-        <x:v>D61-D66</x:v>
+        <x:v>D46-D60</x:v>
       </x:c>
       <x:c r="D17" s="46" t="str">
-        <x:v>复核价格、门店、售后等动态信息</x:v>
+        <x:v>补全P1内链、元数据和结构化数据</x:v>
       </x:c>
       <x:c r="E17" s="46" t="str">
-        <x:v>动态信息复核记录</x:v>
+        <x:v>P1发布包</x:v>
       </x:c>
       <x:c r="F17" s="46" t="str">
-        <x:v>官方渠道</x:v>
+        <x:v>P1页面</x:v>
       </x:c>
       <x:c r="G17" s="46" t="str">
-        <x:v>信源核验</x:v>
+        <x:v>网站编辑</x:v>
       </x:c>
       <x:c r="H17" s="46" t="str">
-        <x:v>记录核验日期</x:v>
+        <x:v>无孤立页、无失效内链</x:v>
       </x:c>
       <x:c r="I17" s="55" t="n">
-        <x:v>46280</x:v>
+        <x:v>46265</x:v>
       </x:c>
       <x:c r="J17" s="55" t="n">
-        <x:v>46285</x:v>
+        <x:v>46279</x:v>
       </x:c>
       <x:c r="K17" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L17" s="47" t="str">
-        <x:v>不补造实时状态</x:v>
+        <x:v>发布前质检</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="45" t="str">
-        <x:v>T-014</x:v>
+        <x:v>T-013</x:v>
       </x:c>
       <x:c r="B18" s="46" t="str">
         <x:v>61-90天 复测维护</x:v>
       </x:c>
       <x:c r="C18" s="46" t="str">
-        <x:v>D64-D68</x:v>
+        <x:v>D61-D66</x:v>
       </x:c>
       <x:c r="D18" s="46" t="str">
-        <x:v>冻结10题复测问题与记录模板</x:v>
+        <x:v>复核价格、门店、售后等动态信息</x:v>
       </x:c>
       <x:c r="E18" s="46" t="str">
-        <x:v>50条复测模板</x:v>
+        <x:v>动态信息复核记录</x:v>
       </x:c>
       <x:c r="F18" s="46" t="str">
-        <x:v>Baseline口径</x:v>
+        <x:v>官方渠道</x:v>
       </x:c>
       <x:c r="G18" s="46" t="str">
-        <x:v>数据QA</x:v>
+        <x:v>信源核验</x:v>
       </x:c>
       <x:c r="H18" s="46" t="str">
-        <x:v>字段完整</x:v>
+        <x:v>记录核验日期</x:v>
       </x:c>
       <x:c r="I18" s="55" t="n">
-        <x:v>46283</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="J18" s="55" t="n">
-        <x:v>46287</x:v>
+        <x:v>46285</x:v>
       </x:c>
       <x:c r="K18" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L18" s="47" t="str">
-        <x:v>Baseline/UserIntent分开</x:v>
+        <x:v>不补造实时状态</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="45" t="str">
-        <x:v>T-015</x:v>
+        <x:v>T-KB-002</x:v>
       </x:c>
       <x:c r="B19" s="46" t="str">
         <x:v>61-90天 复测维护</x:v>
       </x:c>
       <x:c r="C19" s="46" t="str">
-        <x:v>D69-D78</x:v>
+        <x:v>D61-D90</x:v>
       </x:c>
       <x:c r="D19" s="46" t="str">
-        <x:v>人工采集10题×5平台复测</x:v>
+        <x:v>知识库月度复核与失效事实处理</x:v>
       </x:c>
       <x:c r="E19" s="46" t="str">
-        <x:v>50条原始回答</x:v>
+        <x:v>版本审核记录+动态信息失效清单</x:v>
       </x:c>
       <x:c r="F19" s="46" t="str">
-        <x:v>平台可访问</x:v>
+        <x:v>独立知识库</x:v>
       </x:c>
       <x:c r="G19" s="46" t="str">
-        <x:v>项目负责人</x:v>
+        <x:v>数据QA+信源核验</x:v>
       </x:c>
       <x:c r="H19" s="46" t="str">
-        <x:v>日期/模型/模式/URL/截图齐全</x:v>
+        <x:v>过期动态信息不作为当前事实</x:v>
       </x:c>
       <x:c r="I19" s="55" t="n">
-        <x:v>46288</x:v>
+        <x:v>46280</x:v>
       </x:c>
       <x:c r="J19" s="55" t="n">
-        <x:v>46297</x:v>
+        <x:v>46309</x:v>
       </x:c>
       <x:c r="K19" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L19" s="47" t="str">
-        <x:v>不伪造未取回数据</x:v>
+        <x:v>与复测报告同步</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="45" t="str">
-        <x:v>T-016</x:v>
+        <x:v>T-014</x:v>
       </x:c>
       <x:c r="B20" s="46" t="str">
         <x:v>61-90天 复测维护</x:v>
       </x:c>
       <x:c r="C20" s="46" t="str">
-        <x:v>D75-D83</x:v>
+        <x:v>D64-D68</x:v>
       </x:c>
       <x:c r="D20" s="46" t="str">
-        <x:v>按原四维规则复评分与校准</x:v>
+        <x:v>冻结10题复测问题与记录模板</x:v>
       </x:c>
       <x:c r="E20" s="46" t="str">
-        <x:v>复测评分表</x:v>
+        <x:v>50条复测模板</x:v>
       </x:c>
       <x:c r="F20" s="46" t="str">
-        <x:v>50条回答</x:v>
+        <x:v>Baseline口径</x:v>
       </x:c>
       <x:c r="G20" s="46" t="str">
         <x:v>数据QA</x:v>
       </x:c>
       <x:c r="H20" s="46" t="str">
-        <x:v>评分0-20且口径一致</x:v>
+        <x:v>字段完整</x:v>
       </x:c>
       <x:c r="I20" s="55" t="n">
-        <x:v>46294</x:v>
+        <x:v>46283</x:v>
       </x:c>
       <x:c r="J20" s="55" t="n">
-        <x:v>46302</x:v>
+        <x:v>46287</x:v>
       </x:c>
       <x:c r="K20" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L20" s="47" t="str">
-        <x:v>疑似单列</x:v>
+        <x:v>Baseline/UserIntent分开</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="45" t="str">
-        <x:v>T-017</x:v>
+        <x:v>T-015</x:v>
       </x:c>
       <x:c r="B21" s="46" t="str">
         <x:v>61-90天 复测维护</x:v>
       </x:c>
       <x:c r="C21" s="46" t="str">
-        <x:v>D82-D88</x:v>
+        <x:v>D69-D78</x:v>
       </x:c>
       <x:c r="D21" s="46" t="str">
-        <x:v>形成前后差异和限制说明</x:v>
+        <x:v>人工采集10题×5平台复测</x:v>
       </x:c>
       <x:c r="E21" s="46" t="str">
-        <x:v>复测差异报告</x:v>
+        <x:v>50条原始回答</x:v>
       </x:c>
       <x:c r="F21" s="46" t="str">
-        <x:v>复测评分</x:v>
+        <x:v>平台可访问</x:v>
       </x:c>
       <x:c r="G21" s="46" t="str">
-        <x:v>内容策略+数据QA</x:v>
+        <x:v>项目负责人</x:v>
       </x:c>
       <x:c r="H21" s="46" t="str">
-        <x:v>只报告可审计差异</x:v>
+        <x:v>日期/模型/模式/URL/截图齐全</x:v>
       </x:c>
       <x:c r="I21" s="55" t="n">
-        <x:v>46301</x:v>
+        <x:v>46288</x:v>
       </x:c>
       <x:c r="J21" s="55" t="n">
-        <x:v>46307</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="K21" s="58" t="str">
         <x:v>待开始</x:v>
       </x:c>
       <x:c r="L21" s="47" t="str">
+        <x:v>不伪造未取回数据</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="45" t="str">
+        <x:v>T-016</x:v>
+      </x:c>
+      <x:c r="B22" s="46" t="str">
+        <x:v>61-90天 复测维护</x:v>
+      </x:c>
+      <x:c r="C22" s="46" t="str">
+        <x:v>D75-D83</x:v>
+      </x:c>
+      <x:c r="D22" s="46" t="str">
+        <x:v>按原四维规则复评分与校准</x:v>
+      </x:c>
+      <x:c r="E22" s="46" t="str">
+        <x:v>复测评分表</x:v>
+      </x:c>
+      <x:c r="F22" s="46" t="str">
+        <x:v>50条回答</x:v>
+      </x:c>
+      <x:c r="G22" s="46" t="str">
+        <x:v>数据QA</x:v>
+      </x:c>
+      <x:c r="H22" s="46" t="str">
+        <x:v>评分0-20且口径一致</x:v>
+      </x:c>
+      <x:c r="I22" s="55" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="J22" s="55" t="n">
+        <x:v>46302</x:v>
+      </x:c>
+      <x:c r="K22" s="58" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="L22" s="47" t="str">
+        <x:v>疑似单列</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="45" t="str">
+        <x:v>T-017</x:v>
+      </x:c>
+      <x:c r="B23" s="46" t="str">
+        <x:v>61-90天 复测维护</x:v>
+      </x:c>
+      <x:c r="C23" s="46" t="str">
+        <x:v>D82-D88</x:v>
+      </x:c>
+      <x:c r="D23" s="46" t="str">
+        <x:v>形成前后差异和限制说明</x:v>
+      </x:c>
+      <x:c r="E23" s="46" t="str">
+        <x:v>复测差异报告</x:v>
+      </x:c>
+      <x:c r="F23" s="46" t="str">
+        <x:v>复测评分</x:v>
+      </x:c>
+      <x:c r="G23" s="46" t="str">
+        <x:v>内容策略+数据QA</x:v>
+      </x:c>
+      <x:c r="H23" s="46" t="str">
+        <x:v>只报告可审计差异</x:v>
+      </x:c>
+      <x:c r="I23" s="55" t="n">
+        <x:v>46301</x:v>
+      </x:c>
+      <x:c r="J23" s="55" t="n">
+        <x:v>46307</x:v>
+      </x:c>
+      <x:c r="K23" s="58" t="str">
+        <x:v>待开始</x:v>
+      </x:c>
+      <x:c r="L23" s="47" t="str">
         <x:v>不声称因果</x:v>
       </x:c>
     </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="48" t="str">
+    <x:row r="24">
+      <x:c r="A24" s="48" t="str">
         <x:v>T-018</x:v>
       </x:c>
-      <x:c r="B22" s="49" t="str">
+      <x:c r="B24" s="49" t="str">
         <x:v>61-90天 复测维护</x:v>
       </x:c>
-      <x:c r="C22" s="49" t="str">
+      <x:c r="C24" s="49" t="str">
         <x:v>D89-D90</x:v>
       </x:c>
-      <x:c r="D22" s="49" t="str">
+      <x:c r="D24" s="49" t="str">
         <x:v>建立下一轮P2 backlog</x:v>
       </x:c>
-      <x:c r="E22" s="49" t="str">
+      <x:c r="E24" s="49" t="str">
         <x:v>P2优先级清单</x:v>
       </x:c>
-      <x:c r="F22" s="49" t="str">
+      <x:c r="F24" s="49" t="str">
         <x:v>复测与用户需求</x:v>
       </x:c>
-      <x:c r="G22" s="49" t="str">
+      <x:c r="G24" s="49" t="str">
         <x:v>项目负责人</x:v>
       </x:c>
-      <x:c r="H22" s="49" t="str">
+      <x:c r="H24" s="49" t="str">
         <x:v>任务有负责人和验收</x:v>
       </x:c>
-      <x:c r="I22" s="56" t="n">
+      <x:c r="I24" s="56" t="n">
         <x:v>46308</x:v>
       </x:c>
-      <x:c r="J22" s="56" t="n">
+      <x:c r="J24" s="56" t="n">
         <x:v>46309</x:v>
       </x:c>
-      <x:c r="K22" s="59" t="str">
+      <x:c r="K24" s="59" t="str">
         <x:v>待开始</x:v>
       </x:c>
-      <x:c r="L22" s="50" t="str">
+      <x:c r="L24" s="50" t="str">
         <x:v>产品库/案例/比较</x:v>
       </x:c>
     </x:row>
@@ -6202,19 +6278,19 @@
     <x:mergeCell ref="A1:L1"/>
     <x:mergeCell ref="A2:L2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="K5:K22">
+  <x:conditionalFormatting sqref="K5:K24">
     <x:cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="已完成"/>
     <x:cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="执行中"/>
     <x:cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="阻塞"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="K5:K22">
+    <x:dataValidation type="list" sqref="K5:K24">
       <x:formula1>"已完成,执行中,待开始,阻塞"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b177f5fd0274c7e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra77b1f4c58c84a6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6487,17 +6563,16 @@
         <x:v>硬验收</x:v>
       </x:c>
       <x:c r="B11" s="46" t="str">
-        <x:v>质检通过率</x:v>
-      </x:c>
-      <x:c r="C11" s="61" t="n">
-        <x:f>COUNTIF('发布质检'!$G$5:$G$52,"通过")/COUNTA('发布质检'!$G$5:$G$52)</x:f>
-        <x:v>1</x:v>
+        <x:v>知识库工作表</x:v>
+      </x:c>
+      <x:c r="C11" s="46" t="n">
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D11" s="46" t="n">
-        <x:v>1</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E11" s="46" t="str">
-        <x:v>发布质检结果=通过</x:v>
+        <x:v>独立知识库验收</x:v>
       </x:c>
       <x:c r="F11" s="46" t="str">
         <x:f>IF(C11=D11,"通过","待完成")</x:f>
@@ -6507,141 +6582,146 @@
         <x:v>数据QA</x:v>
       </x:c>
       <x:c r="H11" s="46" t="str">
-        <x:v>每次发布</x:v>
+        <x:v>版本发布</x:v>
       </x:c>
       <x:c r="I11" s="46" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="J11" s="47" t="str">
-        <x:v>结构与技术</x:v>
+        <x:v>11表</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="45" t="str">
-        <x:v>观察基线</x:v>
+        <x:v>硬验收</x:v>
       </x:c>
       <x:c r="B12" s="46" t="str">
-        <x:v>品牌识别</x:v>
+        <x:v>信源迁移</x:v>
       </x:c>
       <x:c r="C12" s="46" t="n">
-        <x:v>4.91</x:v>
-      </x:c>
-      <x:c r="D12" s="46" t="str">
-        <x:v>方向性观察</x:v>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="D12" s="46" t="n">
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E12" s="46" t="str">
-        <x:v>Baseline150</x:v>
+        <x:v>独立知识库信源主表</x:v>
       </x:c>
       <x:c r="F12" s="46" t="str">
-        <x:v>基线</x:v>
+        <x:f>IF(C12=D12,"通过","待完成")</x:f>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G12" s="46" t="str">
-        <x:v>数据QA</x:v>
+        <x:v>信源核验</x:v>
       </x:c>
       <x:c r="H12" s="46" t="str">
-        <x:v>复测</x:v>
+        <x:v>版本发布</x:v>
       </x:c>
       <x:c r="I12" s="46" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="J12" s="47" t="str">
-        <x:v>/5</x:v>
+        <x:v>27条</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="45" t="str">
-        <x:v>观察基线</x:v>
+        <x:v>硬验收</x:v>
       </x:c>
       <x:c r="B13" s="46" t="str">
-        <x:v>可靠性</x:v>
+        <x:v>问题知识映射</x:v>
       </x:c>
       <x:c r="C13" s="46" t="n">
-        <x:v>3.69</x:v>
-      </x:c>
-      <x:c r="D13" s="46" t="str">
-        <x:v>方向性观察</x:v>
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D13" s="46" t="n">
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E13" s="46" t="str">
-        <x:v>Baseline150</x:v>
+        <x:v>独立知识库内容FAQ映射</x:v>
       </x:c>
       <x:c r="F13" s="46" t="str">
-        <x:v>基线</x:v>
+        <x:f>IF(C13=D13,"通过","待完成")</x:f>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G13" s="46" t="str">
-        <x:v>数据QA</x:v>
+        <x:v>内容策略+数据QA</x:v>
       </x:c>
       <x:c r="H13" s="46" t="str">
-        <x:v>复测</x:v>
+        <x:v>版本发布</x:v>
       </x:c>
       <x:c r="I13" s="46" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="J13" s="47" t="str">
-        <x:v>/5</x:v>
+        <x:v>30/30</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="45" t="str">
-        <x:v>观察基线</x:v>
+        <x:v>硬验收</x:v>
       </x:c>
       <x:c r="B14" s="46" t="str">
-        <x:v>有效来源覆盖</x:v>
-      </x:c>
-      <x:c r="C14" s="61" t="n">
-        <x:v>0.107</x:v>
-      </x:c>
-      <x:c r="D14" s="46" t="str">
-        <x:v>方向性观察</x:v>
+        <x:v>FAQ事实映射</x:v>
+      </x:c>
+      <x:c r="C14" s="46" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D14" s="46" t="n">
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E14" s="46" t="str">
-        <x:v>16/150</x:v>
+        <x:v>独立知识库内容FAQ映射</x:v>
       </x:c>
       <x:c r="F14" s="46" t="str">
-        <x:v>基线</x:v>
+        <x:f>IF(C14=D14,"通过","待完成")</x:f>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G14" s="46" t="str">
-        <x:v>数据QA</x:v>
+        <x:v>内容策略+信源核验</x:v>
       </x:c>
       <x:c r="H14" s="46" t="str">
-        <x:v>复测</x:v>
+        <x:v>版本发布</x:v>
       </x:c>
       <x:c r="I14" s="46" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="J14" s="47" t="str">
-        <x:v>Baseline</x:v>
+        <x:v>15/15</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="45" t="str">
-        <x:v>观察基线</x:v>
+        <x:v>硬验收</x:v>
       </x:c>
       <x:c r="B15" s="46" t="str">
-        <x:v>非品牌自然提及</x:v>
+        <x:v>质检通过率</x:v>
       </x:c>
       <x:c r="C15" s="61" t="n">
-        <x:v>0.667</x:v>
-      </x:c>
-      <x:c r="D15" s="46" t="str">
-        <x:v>方向性观察</x:v>
+        <x:f>COUNTIF('发布质检'!$G$5:$G$58,"通过")/COUNTA('发布质检'!$G$5:$G$58)</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D15" s="46" t="n">
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="46" t="str">
-        <x:v>20/30</x:v>
+        <x:v>发布质检结果=通过</x:v>
       </x:c>
       <x:c r="F15" s="46" t="str">
-        <x:v>基线</x:v>
+        <x:f>IF(C15=D15,"通过","待完成")</x:f>
+        <x:v>通过</x:v>
       </x:c>
       <x:c r="G15" s="46" t="str">
         <x:v>数据QA</x:v>
       </x:c>
       <x:c r="H15" s="46" t="str">
-        <x:v>复测</x:v>
+        <x:v>每次发布</x:v>
       </x:c>
       <x:c r="I15" s="46" t="str">
-        <x:v>否</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="J15" s="47" t="str">
-        <x:v>UserIntent子样本</x:v>
+        <x:v>结构与技术</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -6649,16 +6729,16 @@
         <x:v>观察基线</x:v>
       </x:c>
       <x:c r="B16" s="46" t="str">
-        <x:v>确认幻觉</x:v>
-      </x:c>
-      <x:c r="C16" s="61" t="n">
-        <x:v>0.093</x:v>
+        <x:v>品牌识别</x:v>
+      </x:c>
+      <x:c r="C16" s="46" t="n">
+        <x:v>4.91</x:v>
       </x:c>
       <x:c r="D16" s="46" t="str">
-        <x:v>分组观察</x:v>
+        <x:v>方向性观察</x:v>
       </x:c>
       <x:c r="E16" s="46" t="str">
-        <x:v>14/150</x:v>
+        <x:v>Baseline150</x:v>
       </x:c>
       <x:c r="F16" s="46" t="str">
         <x:v>基线</x:v>
@@ -6673,68 +6753,196 @@
         <x:v>否</x:v>
       </x:c>
       <x:c r="J16" s="47" t="str">
+        <x:v>/5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="45" t="str">
+        <x:v>观察基线</x:v>
+      </x:c>
+      <x:c r="B17" s="46" t="str">
+        <x:v>可靠性</x:v>
+      </x:c>
+      <x:c r="C17" s="46" t="n">
+        <x:v>3.69</x:v>
+      </x:c>
+      <x:c r="D17" s="46" t="str">
+        <x:v>方向性观察</x:v>
+      </x:c>
+      <x:c r="E17" s="46" t="str">
+        <x:v>Baseline150</x:v>
+      </x:c>
+      <x:c r="F17" s="46" t="str">
+        <x:v>基线</x:v>
+      </x:c>
+      <x:c r="G17" s="46" t="str">
+        <x:v>数据QA</x:v>
+      </x:c>
+      <x:c r="H17" s="46" t="str">
+        <x:v>复测</x:v>
+      </x:c>
+      <x:c r="I17" s="46" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J17" s="47" t="str">
+        <x:v>/5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="45" t="str">
+        <x:v>观察基线</x:v>
+      </x:c>
+      <x:c r="B18" s="46" t="str">
+        <x:v>有效来源覆盖</x:v>
+      </x:c>
+      <x:c r="C18" s="61" t="n">
+        <x:v>0.107</x:v>
+      </x:c>
+      <x:c r="D18" s="46" t="str">
+        <x:v>方向性观察</x:v>
+      </x:c>
+      <x:c r="E18" s="46" t="str">
+        <x:v>16/150</x:v>
+      </x:c>
+      <x:c r="F18" s="46" t="str">
+        <x:v>基线</x:v>
+      </x:c>
+      <x:c r="G18" s="46" t="str">
+        <x:v>数据QA</x:v>
+      </x:c>
+      <x:c r="H18" s="46" t="str">
+        <x:v>复测</x:v>
+      </x:c>
+      <x:c r="I18" s="46" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J18" s="47" t="str">
         <x:v>Baseline</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="48" t="str">
+    <x:row r="19">
+      <x:c r="A19" s="45" t="str">
         <x:v>观察基线</x:v>
       </x:c>
-      <x:c r="B17" s="49" t="str">
+      <x:c r="B19" s="46" t="str">
+        <x:v>非品牌自然提及</x:v>
+      </x:c>
+      <x:c r="C19" s="61" t="n">
+        <x:v>0.667</x:v>
+      </x:c>
+      <x:c r="D19" s="46" t="str">
+        <x:v>方向性观察</x:v>
+      </x:c>
+      <x:c r="E19" s="46" t="str">
+        <x:v>20/30</x:v>
+      </x:c>
+      <x:c r="F19" s="46" t="str">
+        <x:v>基线</x:v>
+      </x:c>
+      <x:c r="G19" s="46" t="str">
+        <x:v>数据QA</x:v>
+      </x:c>
+      <x:c r="H19" s="46" t="str">
+        <x:v>复测</x:v>
+      </x:c>
+      <x:c r="I19" s="46" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J19" s="47" t="str">
+        <x:v>UserIntent子样本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="45" t="str">
+        <x:v>观察基线</x:v>
+      </x:c>
+      <x:c r="B20" s="46" t="str">
+        <x:v>确认幻觉</x:v>
+      </x:c>
+      <x:c r="C20" s="61" t="n">
+        <x:v>0.093</x:v>
+      </x:c>
+      <x:c r="D20" s="46" t="str">
+        <x:v>分组观察</x:v>
+      </x:c>
+      <x:c r="E20" s="46" t="str">
+        <x:v>14/150</x:v>
+      </x:c>
+      <x:c r="F20" s="46" t="str">
+        <x:v>基线</x:v>
+      </x:c>
+      <x:c r="G20" s="46" t="str">
+        <x:v>数据QA</x:v>
+      </x:c>
+      <x:c r="H20" s="46" t="str">
+        <x:v>复测</x:v>
+      </x:c>
+      <x:c r="I20" s="46" t="str">
+        <x:v>否</x:v>
+      </x:c>
+      <x:c r="J20" s="47" t="str">
+        <x:v>Baseline</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="48" t="str">
+        <x:v>观察基线</x:v>
+      </x:c>
+      <x:c r="B21" s="49" t="str">
         <x:v>UserIntent确认幻觉</x:v>
       </x:c>
-      <x:c r="C17" s="62" t="n">
+      <x:c r="C21" s="62" t="n">
         <x:v>0.427</x:v>
       </x:c>
-      <x:c r="D17" s="49" t="str">
+      <x:c r="D21" s="49" t="str">
         <x:v>分组观察</x:v>
       </x:c>
-      <x:c r="E17" s="49" t="str">
+      <x:c r="E21" s="49" t="str">
         <x:v>32/75</x:v>
       </x:c>
-      <x:c r="F17" s="49" t="str">
+      <x:c r="F21" s="49" t="str">
         <x:v>基线</x:v>
       </x:c>
-      <x:c r="G17" s="49" t="str">
+      <x:c r="G21" s="49" t="str">
         <x:v>数据QA</x:v>
       </x:c>
-      <x:c r="H17" s="49" t="str">
+      <x:c r="H21" s="49" t="str">
         <x:v>复测</x:v>
       </x:c>
-      <x:c r="I17" s="49" t="str">
+      <x:c r="I21" s="49" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="J17" s="50" t="str">
+      <x:c r="J21" s="50" t="str">
         <x:v>不得与Baseline混排</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="34" customHeight="1">
-      <x:c r="A20" s="65" t="str">
-        <x:v>指标解释：硬验收=可控制的内容与技术质量；观察基线=只能通过同口径复测观察变化，不作为曝光、销售或AI收录承诺。</x:v>
-      </x:c>
-      <x:c r="B20" s="65"/>
-      <x:c r="C20" s="65"/>
-      <x:c r="D20" s="65"/>
-      <x:c r="E20" s="65"/>
-      <x:c r="F20" s="65"/>
-      <x:c r="G20" s="65"/>
-      <x:c r="H20" s="65"/>
-      <x:c r="I20" s="65"/>
-      <x:c r="J20" s="65"/>
+    <x:row r="24" ht="40" customHeight="1">
+      <x:c r="A24" s="65" t="str">
+        <x:v>指标解释：硬验收=可控制的内容与技术质量；观察基线=只能通过同口径复测观察变化，不作为曝光、销售或AI收录承诺。知识库为独立工作簿和公开JSON，不合并进执行大表。</x:v>
+      </x:c>
+      <x:c r="B24" s="65"/>
+      <x:c r="C24" s="65"/>
+      <x:c r="D24" s="65"/>
+      <x:c r="E24" s="65"/>
+      <x:c r="F24" s="65"/>
+      <x:c r="G24" s="65"/>
+      <x:c r="H24" s="65"/>
+      <x:c r="I24" s="65"/>
+      <x:c r="J24" s="65"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
     <x:mergeCell ref="A2:J2"/>
-    <x:mergeCell ref="A20:J20"/>
+    <x:mergeCell ref="A24:J24"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="F5:F11">
+  <x:conditionalFormatting sqref="F5:F15">
     <x:cfRule type="containsText" dxfId="13" priority="1" operator="containsText" text="通过"/>
     <x:cfRule type="containsText" dxfId="14" priority="2" operator="containsText" text="待"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e7949edde4a45a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R463ac68a8e05459b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8277,25 +8485,25 @@
         <x:v>QA-043</x:v>
       </x:c>
       <x:c r="B47" s="46" t="str">
-        <x:v>站点全局</x:v>
+        <x:v>企业知识库</x:v>
       </x:c>
       <x:c r="C47" s="46" t="str">
-        <x:v>技术</x:v>
+        <x:v>知识库</x:v>
       </x:c>
       <x:c r="D47" s="46" t="str">
-        <x:v>无需登录</x:v>
+        <x:v>直接答案</x:v>
       </x:c>
       <x:c r="E47" s="46" t="str">
-        <x:v>公开链接可直接访问</x:v>
+        <x:v>首屏先给结论</x:v>
       </x:c>
       <x:c r="F47" s="46" t="str">
-        <x:v>浏览器/部署检查</x:v>
+        <x:v>页面结构/源码检查</x:v>
       </x:c>
       <x:c r="G47" s="58" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="H47" s="46" t="str">
-        <x:v>/</x:v>
+        <x:v>/knowledge-base</x:v>
       </x:c>
       <x:c r="I47" s="46" t="str">
         <x:v>网站编辑+数据QA</x:v>
@@ -8304,7 +8512,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K47" s="47" t="str">
-        <x:v>部署后复核</x:v>
+        <x:v>结构验收</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -8312,25 +8520,25 @@
         <x:v>QA-044</x:v>
       </x:c>
       <x:c r="B48" s="46" t="str">
-        <x:v>站点全局</x:v>
+        <x:v>企业知识库</x:v>
       </x:c>
       <x:c r="C48" s="46" t="str">
-        <x:v>技术</x:v>
+        <x:v>知识库</x:v>
       </x:c>
       <x:c r="D48" s="46" t="str">
-        <x:v>响应式</x:v>
+        <x:v>来源</x:v>
       </x:c>
       <x:c r="E48" s="46" t="str">
-        <x:v>电脑和手机端可读</x:v>
+        <x:v>有具体source_id/URL或明确待补</x:v>
       </x:c>
       <x:c r="F48" s="46" t="str">
-        <x:v>响应式布局检查</x:v>
+        <x:v>页面结构/源码检查</x:v>
       </x:c>
       <x:c r="G48" s="58" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="H48" s="46" t="str">
-        <x:v>/</x:v>
+        <x:v>/knowledge-base</x:v>
       </x:c>
       <x:c r="I48" s="46" t="str">
         <x:v>网站编辑+数据QA</x:v>
@@ -8339,7 +8547,7 @@
         <x:v>2026-07-17</x:v>
       </x:c>
       <x:c r="K48" s="47" t="str">
-        <x:v>不溢出</x:v>
+        <x:v>结构验收</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -8347,91 +8555,95 @@
         <x:v>QA-045</x:v>
       </x:c>
       <x:c r="B49" s="46" t="str">
-        <x:v>站点全局</x:v>
+        <x:v>企业知识库</x:v>
       </x:c>
       <x:c r="C49" s="46" t="str">
-        <x:v>技术</x:v>
+        <x:v>知识库</x:v>
       </x:c>
       <x:c r="D49" s="46" t="str">
-        <x:v>robots</x:v>
+        <x:v>事实边界</x:v>
       </x:c>
       <x:c r="E49" s="46" t="str">
-        <x:v>允许基础抓取并指向sitemap</x:v>
+        <x:v>不确定项和禁止表达可见</x:v>
       </x:c>
       <x:c r="F49" s="46" t="str">
-        <x:v>文件检查</x:v>
+        <x:v>页面结构/源码检查</x:v>
       </x:c>
       <x:c r="G49" s="58" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="H49" s="46" t="str">
-        <x:v>/robots.txt</x:v>
+        <x:v>/knowledge-base</x:v>
       </x:c>
       <x:c r="I49" s="46" t="str">
-        <x:v>网站编辑</x:v>
+        <x:v>网站编辑+数据QA</x:v>
       </x:c>
       <x:c r="J49" s="55" t="str">
         <x:v>2026-07-17</x:v>
       </x:c>
-      <x:c r="K49" s="47" t="str"/>
+      <x:c r="K49" s="47" t="str">
+        <x:v>结构验收</x:v>
+      </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="45" t="str">
         <x:v>QA-046</x:v>
       </x:c>
       <x:c r="B50" s="46" t="str">
-        <x:v>站点全局</x:v>
+        <x:v>企业知识库</x:v>
       </x:c>
       <x:c r="C50" s="46" t="str">
-        <x:v>技术</x:v>
+        <x:v>知识库</x:v>
       </x:c>
       <x:c r="D50" s="46" t="str">
-        <x:v>sitemap</x:v>
+        <x:v>更新时间</x:v>
       </x:c>
       <x:c r="E50" s="46" t="str">
-        <x:v>包含策略页和核心内容页</x:v>
+        <x:v>页面显示更新时间</x:v>
       </x:c>
       <x:c r="F50" s="46" t="str">
-        <x:v>文件检查</x:v>
+        <x:v>页面结构/源码检查</x:v>
       </x:c>
       <x:c r="G50" s="58" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="H50" s="46" t="str">
-        <x:v>/sitemap.xml</x:v>
+        <x:v>/knowledge-base</x:v>
       </x:c>
       <x:c r="I50" s="46" t="str">
-        <x:v>网站编辑</x:v>
+        <x:v>网站编辑+数据QA</x:v>
       </x:c>
       <x:c r="J50" s="55" t="str">
         <x:v>2026-07-17</x:v>
       </x:c>
-      <x:c r="K50" s="47" t="str"/>
+      <x:c r="K50" s="47" t="str">
+        <x:v>结构验收</x:v>
+      </x:c>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="45" t="str">
         <x:v>QA-047</x:v>
       </x:c>
       <x:c r="B51" s="46" t="str">
-        <x:v>站点全局</x:v>
+        <x:v>企业知识库</x:v>
       </x:c>
       <x:c r="C51" s="46" t="str">
-        <x:v>交付</x:v>
+        <x:v>知识库</x:v>
       </x:c>
       <x:c r="D51" s="46" t="str">
-        <x:v>下载入口</x:v>
+        <x:v>内部链接</x:v>
       </x:c>
       <x:c r="E51" s="46" t="str">
-        <x:v>DOCX/PDF/XLSX均可下载</x:v>
+        <x:v>至少2个相关页面</x:v>
       </x:c>
       <x:c r="F51" s="46" t="str">
-        <x:v>链接检查</x:v>
+        <x:v>页面结构/源码检查</x:v>
       </x:c>
       <x:c r="G51" s="58" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="H51" s="46" t="str">
-        <x:v>/strategy</x:v>
+        <x:v>/knowledge-base</x:v>
       </x:c>
       <x:c r="I51" s="46" t="str">
         <x:v>网站编辑+数据QA</x:v>
@@ -8439,58 +8651,246 @@
       <x:c r="J51" s="55" t="str">
         <x:v>2026-07-17</x:v>
       </x:c>
-      <x:c r="K51" s="47" t="str"/>
+      <x:c r="K51" s="47" t="str">
+        <x:v>结构验收</x:v>
+      </x:c>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="48" t="str">
+      <x:c r="A52" s="45" t="str">
         <x:v>QA-048</x:v>
       </x:c>
-      <x:c r="B52" s="49" t="str">
+      <x:c r="B52" s="46" t="str">
+        <x:v>企业知识库</x:v>
+      </x:c>
+      <x:c r="C52" s="46" t="str">
+        <x:v>知识库</x:v>
+      </x:c>
+      <x:c r="D52" s="46" t="str">
+        <x:v>元数据</x:v>
+      </x:c>
+      <x:c r="E52" s="46" t="str">
+        <x:v>title与description准确</x:v>
+      </x:c>
+      <x:c r="F52" s="46" t="str">
+        <x:v>页面结构/源码检查</x:v>
+      </x:c>
+      <x:c r="G52" s="58" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="H52" s="46" t="str">
+        <x:v>/knowledge-base</x:v>
+      </x:c>
+      <x:c r="I52" s="46" t="str">
+        <x:v>网站编辑+数据QA</x:v>
+      </x:c>
+      <x:c r="J52" s="55" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K52" s="47" t="str">
+        <x:v>结构验收</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="45" t="str">
+        <x:v>QA-049</x:v>
+      </x:c>
+      <x:c r="B53" s="46" t="str">
         <x:v>站点全局</x:v>
       </x:c>
-      <x:c r="C52" s="49" t="str">
+      <x:c r="C53" s="46" t="str">
+        <x:v>技术</x:v>
+      </x:c>
+      <x:c r="D53" s="46" t="str">
+        <x:v>无需登录</x:v>
+      </x:c>
+      <x:c r="E53" s="46" t="str">
+        <x:v>公开链接可直接访问</x:v>
+      </x:c>
+      <x:c r="F53" s="46" t="str">
+        <x:v>浏览器/部署检查</x:v>
+      </x:c>
+      <x:c r="G53" s="58" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="H53" s="46" t="str">
+        <x:v>/</x:v>
+      </x:c>
+      <x:c r="I53" s="46" t="str">
+        <x:v>网站编辑+数据QA</x:v>
+      </x:c>
+      <x:c r="J53" s="55" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K53" s="47" t="str">
+        <x:v>部署后复核</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="45" t="str">
+        <x:v>QA-050</x:v>
+      </x:c>
+      <x:c r="B54" s="46" t="str">
+        <x:v>站点全局</x:v>
+      </x:c>
+      <x:c r="C54" s="46" t="str">
+        <x:v>技术</x:v>
+      </x:c>
+      <x:c r="D54" s="46" t="str">
+        <x:v>响应式</x:v>
+      </x:c>
+      <x:c r="E54" s="46" t="str">
+        <x:v>电脑和手机端可读</x:v>
+      </x:c>
+      <x:c r="F54" s="46" t="str">
+        <x:v>响应式布局检查</x:v>
+      </x:c>
+      <x:c r="G54" s="58" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="H54" s="46" t="str">
+        <x:v>/</x:v>
+      </x:c>
+      <x:c r="I54" s="46" t="str">
+        <x:v>网站编辑+数据QA</x:v>
+      </x:c>
+      <x:c r="J54" s="55" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K54" s="47" t="str">
+        <x:v>不溢出</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="45" t="str">
+        <x:v>QA-051</x:v>
+      </x:c>
+      <x:c r="B55" s="46" t="str">
+        <x:v>站点全局</x:v>
+      </x:c>
+      <x:c r="C55" s="46" t="str">
+        <x:v>技术</x:v>
+      </x:c>
+      <x:c r="D55" s="46" t="str">
+        <x:v>robots</x:v>
+      </x:c>
+      <x:c r="E55" s="46" t="str">
+        <x:v>允许基础抓取并指向sitemap</x:v>
+      </x:c>
+      <x:c r="F55" s="46" t="str">
+        <x:v>文件检查</x:v>
+      </x:c>
+      <x:c r="G55" s="58" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="H55" s="46" t="str">
+        <x:v>/robots.txt</x:v>
+      </x:c>
+      <x:c r="I55" s="46" t="str">
+        <x:v>网站编辑</x:v>
+      </x:c>
+      <x:c r="J55" s="55" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K55" s="47" t="str"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="45" t="str">
+        <x:v>QA-052</x:v>
+      </x:c>
+      <x:c r="B56" s="46" t="str">
+        <x:v>站点全局</x:v>
+      </x:c>
+      <x:c r="C56" s="46" t="str">
+        <x:v>技术</x:v>
+      </x:c>
+      <x:c r="D56" s="46" t="str">
+        <x:v>sitemap</x:v>
+      </x:c>
+      <x:c r="E56" s="46" t="str">
+        <x:v>包含策略页和核心内容页</x:v>
+      </x:c>
+      <x:c r="F56" s="46" t="str">
+        <x:v>文件检查</x:v>
+      </x:c>
+      <x:c r="G56" s="58" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="H56" s="46" t="str">
+        <x:v>/sitemap.xml</x:v>
+      </x:c>
+      <x:c r="I56" s="46" t="str">
+        <x:v>网站编辑</x:v>
+      </x:c>
+      <x:c r="J56" s="55" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K56" s="47" t="str"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="45" t="str">
+        <x:v>QA-053</x:v>
+      </x:c>
+      <x:c r="B57" s="46" t="str">
+        <x:v>站点全局</x:v>
+      </x:c>
+      <x:c r="C57" s="46" t="str">
+        <x:v>交付</x:v>
+      </x:c>
+      <x:c r="D57" s="46" t="str">
+        <x:v>下载入口</x:v>
+      </x:c>
+      <x:c r="E57" s="46" t="str">
+        <x:v>DOCX/PDF/XLSX均可下载</x:v>
+      </x:c>
+      <x:c r="F57" s="46" t="str">
+        <x:v>链接检查</x:v>
+      </x:c>
+      <x:c r="G57" s="58" t="str">
+        <x:v>通过</x:v>
+      </x:c>
+      <x:c r="H57" s="46" t="str">
+        <x:v>/strategy</x:v>
+      </x:c>
+      <x:c r="I57" s="46" t="str">
+        <x:v>网站编辑+数据QA</x:v>
+      </x:c>
+      <x:c r="J57" s="55" t="str">
+        <x:v>2026-07-17</x:v>
+      </x:c>
+      <x:c r="K57" s="47" t="str"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="48" t="str">
+        <x:v>QA-054</x:v>
+      </x:c>
+      <x:c r="B58" s="49" t="str">
+        <x:v>站点全局</x:v>
+      </x:c>
+      <x:c r="C58" s="49" t="str">
         <x:v>声明</x:v>
       </x:c>
-      <x:c r="D52" s="49" t="str">
+      <x:c r="D58" s="49" t="str">
         <x:v>研究边界</x:v>
       </x:c>
-      <x:c r="E52" s="49" t="str">
+      <x:c r="E58" s="49" t="str">
         <x:v>不代表官方、不声称效果提升</x:v>
       </x:c>
-      <x:c r="F52" s="49" t="str">
+      <x:c r="F58" s="49" t="str">
         <x:v>文案检查</x:v>
       </x:c>
-      <x:c r="G52" s="59" t="str">
+      <x:c r="G58" s="59" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="H52" s="49" t="str">
+      <x:c r="H58" s="49" t="str">
         <x:v>/strategy</x:v>
       </x:c>
-      <x:c r="I52" s="49" t="str">
+      <x:c r="I58" s="49" t="str">
         <x:v>内容策略+数据QA</x:v>
       </x:c>
-      <x:c r="J52" s="56" t="str">
+      <x:c r="J58" s="56" t="str">
         <x:v>2026-07-17</x:v>
       </x:c>
-      <x:c r="K52" s="50" t="str"/>
-    </x:row>
-    <x:row r="53">
-      <x:c r="J53" s="60"/>
-    </x:row>
-    <x:row r="54">
-      <x:c r="J54" s="60"/>
-    </x:row>
-    <x:row r="55">
-      <x:c r="J55" s="60"/>
-    </x:row>
-    <x:row r="56">
-      <x:c r="J56" s="60"/>
-    </x:row>
-    <x:row r="57">
-      <x:c r="J57" s="60"/>
-    </x:row>
-    <x:row r="58">
-      <x:c r="J58" s="60"/>
+      <x:c r="K58" s="50" t="str"/>
     </x:row>
     <x:row r="59">
       <x:c r="J59" s="60"/>
@@ -8623,19 +9023,19 @@
     <x:mergeCell ref="A1:K1"/>
     <x:mergeCell ref="A2:K2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="G5:G52">
+  <x:conditionalFormatting sqref="G5:G58">
     <x:cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="通过"/>
     <x:cfRule type="containsText" dxfId="11" priority="2" operator="containsText" text="待"/>
     <x:cfRule type="containsText" dxfId="12" priority="3" operator="containsText" text="不通过"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="G5:G52">
+    <x:dataValidation type="list" sqref="G5:G58">
       <x:formula1>"通过,待复核,不通过,不适用"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde357a8da1c24c3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c0bbe144b03464c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>